<commit_message>
Update admin UI: Add categories and brands dropdowns, setup ProductManager
</commit_message>
<xml_diff>
--- a/public/plantilla_productos.xlsx
+++ b/public/plantilla_productos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,18 +407,24 @@
         <v>Nombre</v>
       </c>
       <c r="C1" t="str">
+        <v>Marca</v>
+      </c>
+      <c r="D1" t="str">
         <v>Categoría</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
+        <v>Subcategoría</v>
+      </c>
+      <c r="F1" t="str">
         <v>Precio</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Stock</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Descripción</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Imagen</v>
       </c>
     </row>
@@ -430,18 +436,24 @@
         <v>Fender Stratocaster American Pro II</v>
       </c>
       <c r="C2" t="str">
+        <v>Fender</v>
+      </c>
+      <c r="D2" t="str">
         <v>Guitarras Eléctricas</v>
       </c>
-      <c r="D2">
+      <c r="E2" t="str">
+        <v>Stratocaster</v>
+      </c>
+      <c r="F2">
         <v>1850000</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>3</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>Guitarra eléctrica con mástil Deep C y pastillas V-Mod II.</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v/>
       </c>
     </row>
@@ -453,24 +465,30 @@
         <v>Boss DS-1 Distortion</v>
       </c>
       <c r="C3" t="str">
+        <v>Boss</v>
+      </c>
+      <c r="D3" t="str">
         <v>Pedales y Accesorios</v>
       </c>
-      <c r="D3">
+      <c r="E3" t="str">
+        <v>Pedales de Distorsión</v>
+      </c>
+      <c r="F3">
         <v>120000</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>15</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
         <v>El clásico pedal de distorsión utilizado por leyendas del rock.</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>